<commit_message>
docs+ui: record client-confirmed project names; spacing for contact-card links
- projects-inventory.xlsx and AUDIT_REPORT §7.3 mirror: English names of
  projects 1, 2, 5, 6, 18, 24, 27 marked confirmed by client (2026-09-15)
- contact card links (e.g. "View on map") get icon/text spacing

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MESxPkpNmdXTMecbaPtRf5
</commit_message>
<xml_diff>
--- a/docs/projects-inventory.xlsx
+++ b/docs/projects-inventory.xlsx
@@ -39,10 +39,10 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00006100"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00006100"/>
     </font>
   </fonts>
   <fills count="7">
@@ -64,12 +64,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -118,25 +118,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -579,14 +579,14 @@
           <t>Asyut Western Road - Asyut Gate October</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>(unchanged — client to confirm)</t>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Asyut Western Road – October Gate, Asyut (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Yes — "بوابة أسيوط أكتوبر" rendered as "Asyut Gate October"; meaning/word order unclear. Confirm intended English.</t>
+          <t>Yes — "بوابة أسيوط أكتوبر" rendered as "Asyut Gate October"; meaning/word order unclear. Confirm intended English. → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -594,7 +594,7 @@
           <t>../imgs/slider.jpg</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -606,7 +606,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish. Confirm English name. Also confirm whether unused imgs/slider1–3.jpg belong to this project (HTML references "slider.jpg").</t>
+          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish. Also confirm whether unused imgs/slider1–3.jpg belong to this project (HTML references "slider.jpg").</t>
         </is>
       </c>
     </row>
@@ -624,14 +624,14 @@
           <t>Asyut Western Road - Fayoum Silos &amp; Checkpoint</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>(unchanged — client to confirm)</t>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Asyut Western Road – Fayoum Silos &amp; Traffic Checkpoint (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Yes — "مرور الفيوم" (Fayoum traffic point) rendered as "Checkpoint"; Arabic word order (Silos, then Fayoum traffic) differs. Confirm wording.</t>
+          <t>Yes — "مرور الفيوم" (Fayoum traffic point) rendered as "Checkpoint"; Arabic word order (Silos, then Fayoum traffic) differs. Confirm wording. → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -639,7 +639,7 @@
           <t>../imgs/project2.jpg</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -651,7 +651,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish. Confirm English name.</t>
+          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish.</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
           <t>../imgs/project3.jpg</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -729,7 +729,7 @@
           <t>../imgs/project8.jpg</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -759,14 +759,14 @@
           <t>Future of Egypt Project</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>(unchanged — client to confirm)</t>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Future of Egypt Project (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>No — optional: confirm whether the client prefers a transliterated official name.</t>
+          <t>No — optional: confirm whether the client prefers a transliterated official name. → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -774,7 +774,7 @@
           <t>../imgs/مستقبل_مصر.jpg</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -804,14 +804,14 @@
           <t>Talbia Axis</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>(unchanged — client to confirm)</t>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Talbia Axis (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>No — transliteration variant ("Talbia" / "Talbiya"); confirm preferred spelling.</t>
+          <t>No — transliteration variant ("Talbia" / "Talbiya"); confirm preferred spelling. → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -819,7 +819,7 @@
           <t>../imgs/project4.jpg</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -864,7 +864,7 @@
           <t>../imgs/project5.jpg</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -909,7 +909,7 @@
           <t>../imgs/project9.jpg</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -954,7 +954,7 @@
           <t>../imgs/محور_عمرو_بنالعاص.jpg</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -984,7 +984,7 @@
           <t>Ring Road Development - Qalyoub Exit</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Ring Road Development &amp; Widening - Qalyoub Exit</t>
         </is>
@@ -999,7 +999,7 @@
           <t>../imgs/project6.jpg</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1029,7 +1029,7 @@
           <t>Ring Road Development - Mansouria Exit</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Ring Road Development &amp; Widening - Mansouria (Haram) Exit</t>
         </is>
@@ -1044,7 +1044,7 @@
           <t>../imgs/project7.jpg</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1074,7 +1074,7 @@
           <t>Ring Road Development - Bahtim</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Ring Road Development &amp; Widening - Bahtim</t>
         </is>
@@ -1089,7 +1089,7 @@
           <t>../imgs/project11.jpg</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1119,7 +1119,7 @@
           <t>Cairo University Roads - Sheikh Zayed Branch</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Cairo University Roads Development &amp; Widening - Sheikh Zayed Branch</t>
         </is>
@@ -1134,7 +1134,7 @@
           <t>../imgs/project12.jpg</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1164,7 +1164,7 @@
           <t>El-Masallat Road - Suez</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>El-Mothallath (Triangle) Road Development &amp; Widening - Suez</t>
         </is>
@@ -1179,7 +1179,7 @@
           <t>../imgs/project13.jpg</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1209,7 +1209,7 @@
           <t>Suez - Sokhna Road</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Suez - Sokhna Road Development &amp; Widening</t>
         </is>
@@ -1224,7 +1224,7 @@
           <t>../imgs/project14.jpg</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1254,7 +1254,7 @@
           <t>October Western Sector Maintenance</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>October Western Sector Development &amp; Maintenance</t>
         </is>
@@ -1269,7 +1269,7 @@
           <t>../imgs/الطريق_الغربي_اكتوبر.jpg</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1299,7 +1299,7 @@
           <t>October Southern Districts Maintenance</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>October Southern Districts Development &amp; Maintenance</t>
         </is>
@@ -1314,7 +1314,7 @@
           <t>../imgs/project16.jpg</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1344,14 +1344,14 @@
           <t>October West Sumed Maintenance</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>October West Sumed Development &amp; Maintenance (transliteration "Sumed" still to confirm)</t>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>October West Sumed Development &amp; Maintenance (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Yes — "سوميد" transliterated as "Sumed"; confirm the spelling the client/owner uses.</t>
+          <t>Yes — "سوميد" transliterated as "Sumed"; confirm the spelling the client/owner uses. → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1359,7 +1359,7 @@
           <t>../imgs/project17.jpg</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish. Confirm English name.</t>
+          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish.</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
           <t>October Northern Sector Maintenance</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>October Northern Sector Development &amp; Maintenance</t>
         </is>
@@ -1404,7 +1404,7 @@
           <t>../imgs/project18.jpg</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1434,7 +1434,7 @@
           <t>Mokattam Maintenance</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Mokattam Development &amp; Maintenance</t>
         </is>
@@ -1449,7 +1449,7 @@
           <t>../imgs/project19.jpg</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1479,7 +1479,7 @@
           <t>Zahraa Maadi Maintenance</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>Zahraa Maadi Development &amp; Maintenance</t>
         </is>
@@ -1494,7 +1494,7 @@
           <t>../imgs/project20.jpg</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1524,7 +1524,7 @@
           <t>Maadi Nerco Maintenance</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Maadi Nerco Development &amp; Maintenance</t>
         </is>
@@ -1539,7 +1539,7 @@
           <t>../imgs/project21.jpg</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1569,7 +1569,7 @@
           <t>Natrn Valley Maintenance</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Wadi El Natrun Development &amp; Maintenance</t>
         </is>
@@ -1584,7 +1584,7 @@
           <t>../imgs/وادي_النطرون.jpg</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1614,14 +1614,14 @@
           <t>Brick Factory - New Capital (R1 &amp; R2)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>(unchanged — client to confirm)</t>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Brick Factory – New Capital (R1 &amp; R2) (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Yes — English adds "New"; Arabic says only "العاصمة" (the Capital). Confirm it is the New Administrative Capital.</t>
+          <t>Yes — English adds "New"; Arabic says only "العاصمة" (the Capital). Confirm it is the New Administrative Capital. → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1629,7 +1629,7 @@
           <t>../imgs/factory1.jpg</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish. Confirm English name.</t>
+          <t>Project photo(s): 1–3 per project, 4:3, min 1200×900, with permission to publish.</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
           <t>../imgs/factory2.jpg</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1719,7 +1719,7 @@
           <t>../imgs/factory3.jpg</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1749,14 +1749,14 @@
           <t>Brick Factory - 15 May City</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>(unchanged — client to confirm)</t>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Brick Factory – 15th of May City (confirmed by client 2026-09-15)</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>No (minor) — commonly written "15th of May City".</t>
+          <t>No (minor) — commonly written "15th of May City". → RESOLVED: English name confirmed by client 2026-09-15.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1764,7 +1764,7 @@
           <t>../imgs/factory4.jpg</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>No – 404</t>
         </is>
@@ -1828,11 +1828,11 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>English names corrected</t>
+          <t>English names corrected or client-confirmed</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>